<commit_message>
Redo Asti Tav. 10: real double reading, 0 validation flags
Re-run with 01b (Senza/TOTALE block location), pass 1 from OCR (01c),
independent visual pass 2 of the strip crops, disagreements decided by
check_pass.py (both block sum and Tav. 1 sum) or by zoomed re-read.
flags_asti.csv is empty; tav10_asti.dta rebuilt from the validated data.
See docs/audit_2026-10.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011mvLWFfLFbnKm7v6S9L2EZ
</commit_message>
<xml_diff>
--- a/output/tav10_asti.xlsx
+++ b/output/tav10_asti.xlsx
@@ -822,61 +822,61 @@
         <v>32</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>2.61</v>
       </c>
       <c r="H2" t="n">
         <v>141</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>23.94</v>
       </c>
       <c r="J2" t="n">
         <v>111</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>29.53</v>
       </c>
       <c r="L2" t="n">
         <v>167</v>
       </c>
       <c r="M2" t="n">
-        <v>0</v>
+        <v>61.88</v>
       </c>
       <c r="N2" t="n">
         <v>104</v>
       </c>
       <c r="O2" t="n">
-        <v>0</v>
+        <v>47.66</v>
       </c>
       <c r="P2" t="n">
         <v>332</v>
       </c>
       <c r="Q2" t="n">
-        <v>0</v>
+        <v>206.26</v>
       </c>
       <c r="R2" t="n">
         <v>435</v>
       </c>
       <c r="S2" t="n">
-        <v>0</v>
+        <v>381.86</v>
       </c>
       <c r="T2" t="n">
         <v>607</v>
       </c>
       <c r="U2" t="n">
-        <v>0</v>
+        <v>760.37</v>
       </c>
       <c r="V2" t="n">
         <v>685</v>
       </c>
       <c r="W2" t="n">
-        <v>0</v>
+        <v>1201.78</v>
       </c>
       <c r="X2" t="n">
         <v>570</v>
       </c>
       <c r="Y2" t="n">
-        <v>0</v>
+        <v>1293.42</v>
       </c>
       <c r="Z2" t="n">
         <v>562</v>
@@ -957,17 +957,17 @@
         <v>478.23</v>
       </c>
       <c r="AZ2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BA2" t="n">
+        <v>265.36</v>
+      </c>
+      <c r="BB2" t="n">
+        <v>3</v>
+      </c>
+      <c r="BC2" t="n">
         <v>172.95</v>
       </c>
-      <c r="BB2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC2" t="n">
-        <v>0</v>
-      </c>
       <c r="BD2" t="n">
         <v>0</v>
       </c>
@@ -1017,7 +1017,7 @@
         <v>0</v>
       </c>
       <c r="BT2" t="n">
-        <v>8522</v>
+        <v>8531</v>
       </c>
       <c r="BU2" t="n">
         <v>36885.46</v>
@@ -1053,7 +1053,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
@@ -1062,16 +1062,16 @@
         <v>57</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>4.88</v>
       </c>
       <c r="H3" t="n">
         <v>348</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>61.31</v>
       </c>
       <c r="J3" t="n">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="K3" t="n">
         <v>79.45</v>
@@ -1086,7 +1086,7 @@
         <v>331</v>
       </c>
       <c r="O3" t="n">
-        <v>154.2</v>
+        <v>154.26</v>
       </c>
       <c r="P3" t="n">
         <v>859</v>
@@ -1158,67 +1158,67 @@
         <v>453</v>
       </c>
       <c r="AM3" t="n">
-        <v>3864.28</v>
+        <v>3882.39</v>
       </c>
       <c r="AN3" t="n">
         <v>154</v>
       </c>
       <c r="AO3" t="n">
-        <v>1706.63</v>
+        <v>1718.29</v>
       </c>
       <c r="AP3" t="n">
         <v>67</v>
       </c>
       <c r="AQ3" t="n">
-        <v>915.08</v>
+        <v>911</v>
       </c>
       <c r="AR3" t="n">
         <v>56</v>
       </c>
       <c r="AS3" t="n">
-        <v>953.52</v>
+        <v>944.2</v>
       </c>
       <c r="AT3" t="n">
         <v>20</v>
       </c>
       <c r="AU3" t="n">
-        <v>447.21</v>
+        <v>447.14</v>
       </c>
       <c r="AV3" t="n">
         <v>8</v>
       </c>
       <c r="AW3" t="n">
-        <v>218.65</v>
+        <v>216.55</v>
       </c>
       <c r="AX3" t="n">
         <v>8</v>
       </c>
       <c r="AY3" t="n">
-        <v>273.26</v>
+        <v>268.68</v>
       </c>
       <c r="AZ3" t="n">
         <v>1</v>
       </c>
       <c r="BA3" t="n">
-        <v>41.5</v>
+        <v>40.8</v>
       </c>
       <c r="BB3" t="n">
         <v>4</v>
       </c>
       <c r="BC3" t="n">
-        <v>245.08</v>
+        <v>224.8</v>
       </c>
       <c r="BD3" t="n">
         <v>3</v>
       </c>
       <c r="BE3" t="n">
-        <v>245</v>
+        <v>256.2</v>
       </c>
       <c r="BF3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BG3" t="n">
-        <v>0</v>
+        <v>119.77</v>
       </c>
       <c r="BH3" t="n">
         <v>0</v>
@@ -1260,7 +1260,7 @@
         <v>15185</v>
       </c>
       <c r="BU3" t="n">
-        <v>45392.98</v>
+        <v>45392.93</v>
       </c>
       <c r="BV3" t="inlineStr">
         <is>
@@ -1293,184 +1293,184 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
+        <v>82</v>
+      </c>
+      <c r="G4" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="H4" t="n">
+        <v>395</v>
+      </c>
+      <c r="I4" t="n">
+        <v>68.18000000000001</v>
+      </c>
+      <c r="J4" t="n">
+        <v>343</v>
+      </c>
+      <c r="K4" t="n">
+        <v>88.86</v>
+      </c>
+      <c r="L4" t="n">
+        <v>557</v>
+      </c>
+      <c r="M4" t="n">
+        <v>203.75</v>
+      </c>
+      <c r="N4" t="n">
+        <v>348</v>
+      </c>
+      <c r="O4" t="n">
+        <v>161.36</v>
+      </c>
+      <c r="P4" t="n">
+        <v>960</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>596.6900000000001</v>
+      </c>
+      <c r="R4" t="n">
+        <v>1149</v>
+      </c>
+      <c r="S4" t="n">
+        <v>1005.87</v>
+      </c>
+      <c r="T4" t="n">
+        <v>1599</v>
+      </c>
+      <c r="U4" t="n">
+        <v>2006.89</v>
+      </c>
+      <c r="V4" t="n">
+        <v>1922</v>
+      </c>
+      <c r="W4" t="n">
+        <v>3391.56</v>
+      </c>
+      <c r="X4" t="n">
+        <v>1465</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>3320.44</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>1384</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>3821.49</v>
+      </c>
+      <c r="AB4" t="n">
+        <v>1045</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>3403.23</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>919</v>
+      </c>
+      <c r="AE4" t="n">
+        <v>3464.18</v>
+      </c>
+      <c r="AF4" t="n">
+        <v>554</v>
+      </c>
+      <c r="AG4" t="n">
+        <v>2359.33</v>
+      </c>
+      <c r="AH4" t="n">
+        <v>524</v>
+      </c>
+      <c r="AI4" t="n">
+        <v>2491.13</v>
+      </c>
+      <c r="AJ4" t="n">
+        <v>1108</v>
+      </c>
+      <c r="AK4" t="n">
+        <v>6674.04</v>
+      </c>
+      <c r="AL4" t="n">
+        <v>345</v>
+      </c>
+      <c r="AM4" t="n">
+        <v>2947.37</v>
+      </c>
+      <c r="AN4" t="n">
+        <v>149</v>
+      </c>
+      <c r="AO4" t="n">
+        <v>1648.71</v>
+      </c>
+      <c r="AP4" t="n">
+        <v>48</v>
+      </c>
+      <c r="AQ4" t="n">
+        <v>656.62</v>
+      </c>
+      <c r="AR4" t="n">
+        <v>47</v>
+      </c>
+      <c r="AS4" t="n">
+        <v>816.9299999999999</v>
+      </c>
+      <c r="AT4" t="n">
+        <v>15</v>
+      </c>
+      <c r="AU4" t="n">
+        <v>333.52</v>
+      </c>
+      <c r="AV4" t="n">
+        <v>5</v>
+      </c>
+      <c r="AW4" t="n">
+        <v>137.52</v>
+      </c>
+      <c r="AX4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY4" t="n">
+        <v>103.27</v>
+      </c>
+      <c r="AZ4" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA4" t="n">
+        <v>122.03</v>
+      </c>
+      <c r="BB4" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC4" t="n">
+        <v>68.43000000000001</v>
+      </c>
+      <c r="BD4" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE4" t="n">
+        <v>78.42</v>
+      </c>
+      <c r="BF4" t="n">
         <v>2</v>
       </c>
-      <c r="G4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" t="n">
-        <v>82</v>
-      </c>
-      <c r="K4" t="n">
-        <v>6.99</v>
-      </c>
-      <c r="L4" t="n">
-        <v>395</v>
-      </c>
-      <c r="M4" t="n">
-        <v>68.18000000000001</v>
-      </c>
-      <c r="N4" t="n">
-        <v>343</v>
-      </c>
-      <c r="O4" t="n">
-        <v>88.86</v>
-      </c>
-      <c r="P4" t="n">
-        <v>557</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>203.75</v>
-      </c>
-      <c r="R4" t="n">
-        <v>348</v>
-      </c>
-      <c r="S4" t="n">
-        <v>161.36</v>
-      </c>
-      <c r="T4" t="n">
-        <v>960</v>
-      </c>
-      <c r="U4" t="n">
-        <v>596.6900000000001</v>
-      </c>
-      <c r="V4" t="n">
-        <v>1149</v>
-      </c>
-      <c r="W4" t="n">
-        <v>1005.87</v>
-      </c>
-      <c r="X4" t="n">
-        <v>1599</v>
-      </c>
-      <c r="Y4" t="n">
-        <v>2006.89</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>1922</v>
-      </c>
-      <c r="AA4" t="n">
-        <v>3391.56</v>
-      </c>
-      <c r="AB4" t="n">
-        <v>1465</v>
-      </c>
-      <c r="AC4" t="n">
-        <v>3320.44</v>
-      </c>
-      <c r="AD4" t="n">
-        <v>1384</v>
-      </c>
-      <c r="AE4" t="n">
-        <v>3821.49</v>
-      </c>
-      <c r="AF4" t="n">
-        <v>1045</v>
-      </c>
-      <c r="AG4" t="n">
-        <v>3403.23</v>
-      </c>
-      <c r="AH4" t="n">
-        <v>919</v>
-      </c>
-      <c r="AI4" t="n">
-        <v>3464.18</v>
-      </c>
-      <c r="AJ4" t="n">
-        <v>554</v>
-      </c>
-      <c r="AK4" t="n">
-        <v>2359.33</v>
-      </c>
-      <c r="AL4" t="n">
-        <v>524</v>
-      </c>
-      <c r="AM4" t="n">
-        <v>2491.13</v>
-      </c>
-      <c r="AN4" t="n">
-        <v>1108</v>
-      </c>
-      <c r="AO4" t="n">
-        <v>6674.04</v>
-      </c>
-      <c r="AP4" t="n">
-        <v>345</v>
-      </c>
-      <c r="AQ4" t="n">
-        <v>2947.37</v>
-      </c>
-      <c r="AR4" t="n">
-        <v>149</v>
-      </c>
-      <c r="AS4" t="n">
-        <v>1648.71</v>
-      </c>
-      <c r="AT4" t="n">
-        <v>48</v>
-      </c>
-      <c r="AU4" t="n">
-        <v>656.62</v>
-      </c>
-      <c r="AV4" t="n">
-        <v>47</v>
-      </c>
-      <c r="AW4" t="n">
-        <v>816.9299999999999</v>
-      </c>
-      <c r="AX4" t="n">
-        <v>15</v>
-      </c>
-      <c r="AY4" t="n">
-        <v>333.52</v>
-      </c>
-      <c r="AZ4" t="n">
-        <v>5</v>
-      </c>
-      <c r="BA4" t="n">
-        <v>137.52</v>
-      </c>
-      <c r="BB4" t="n">
-        <v>3</v>
-      </c>
-      <c r="BC4" t="n">
-        <v>103.27</v>
-      </c>
-      <c r="BD4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE4" t="n">
-        <v>122.03</v>
-      </c>
-      <c r="BF4" t="n">
-        <v>0</v>
-      </c>
       <c r="BG4" t="n">
-        <v>68.43000000000001</v>
+        <v>237.94</v>
       </c>
       <c r="BH4" t="n">
         <v>0</v>
       </c>
       <c r="BI4" t="n">
-        <v>78.42</v>
+        <v>0</v>
       </c>
       <c r="BJ4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BK4" t="n">
-        <v>237.94</v>
+        <v>0</v>
       </c>
       <c r="BL4" t="n">
         <v>0</v>
@@ -1539,166 +1539,166 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>0.71</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>2.45</v>
       </c>
       <c r="J5" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="K5" t="n">
-        <v>0.71</v>
+        <v>4.02</v>
       </c>
       <c r="L5" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="M5" t="n">
-        <v>2.45</v>
+        <v>5.55</v>
       </c>
       <c r="N5" t="n">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="O5" t="n">
-        <v>4.02</v>
+        <v>13.85</v>
       </c>
       <c r="P5" t="n">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.55</v>
+        <v>24.58</v>
       </c>
       <c r="R5" t="n">
-        <v>29</v>
+        <v>51</v>
       </c>
       <c r="S5" t="n">
-        <v>13.85</v>
+        <v>46.26</v>
       </c>
       <c r="T5" t="n">
-        <v>39</v>
+        <v>92</v>
       </c>
       <c r="U5" t="n">
-        <v>24.58</v>
+        <v>119.48</v>
       </c>
       <c r="V5" t="n">
-        <v>51</v>
+        <v>110</v>
       </c>
       <c r="W5" t="n">
-        <v>46.26</v>
+        <v>197.16</v>
       </c>
       <c r="X5" t="n">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="Y5" t="n">
-        <v>119.48</v>
+        <v>207.49</v>
       </c>
       <c r="Z5" t="n">
-        <v>110</v>
+        <v>88</v>
       </c>
       <c r="AA5" t="n">
-        <v>197.16</v>
+        <v>248.57</v>
       </c>
       <c r="AB5" t="n">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="AC5" t="n">
-        <v>207.49</v>
+        <v>328.18</v>
       </c>
       <c r="AD5" t="n">
-        <v>88</v>
+        <v>121</v>
       </c>
       <c r="AE5" t="n">
-        <v>248.57</v>
+        <v>460.69</v>
       </c>
       <c r="AF5" t="n">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="AG5" t="n">
-        <v>328.18</v>
+        <v>413.99</v>
       </c>
       <c r="AH5" t="n">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="AI5" t="n">
-        <v>460.69</v>
+        <v>514.02</v>
       </c>
       <c r="AJ5" t="n">
-        <v>96</v>
+        <v>442</v>
       </c>
       <c r="AK5" t="n">
-        <v>413.99</v>
+        <v>2777.09</v>
       </c>
       <c r="AL5" t="n">
-        <v>108</v>
+        <v>273</v>
       </c>
       <c r="AM5" t="n">
-        <v>514.02</v>
+        <v>2405.11</v>
       </c>
       <c r="AN5" t="n">
-        <v>442</v>
+        <v>149</v>
       </c>
       <c r="AO5" t="n">
-        <v>2777.09</v>
+        <v>1654.97</v>
       </c>
       <c r="AP5" t="n">
-        <v>273</v>
+        <v>69</v>
       </c>
       <c r="AQ5" t="n">
-        <v>2405.11</v>
+        <v>932.36</v>
       </c>
       <c r="AR5" t="n">
-        <v>149</v>
+        <v>69</v>
       </c>
       <c r="AS5" t="n">
-        <v>1654.97</v>
+        <v>1173.78</v>
       </c>
       <c r="AT5" t="n">
-        <v>69</v>
+        <v>32</v>
       </c>
       <c r="AU5" t="n">
-        <v>932.36</v>
+        <v>713.0599999999999</v>
       </c>
       <c r="AV5" t="n">
-        <v>69</v>
+        <v>12</v>
       </c>
       <c r="AW5" t="n">
-        <v>1173.78</v>
+        <v>334.71</v>
       </c>
       <c r="AX5" t="n">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="AY5" t="n">
-        <v>713.0599999999999</v>
+        <v>367.1</v>
       </c>
       <c r="AZ5" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="BA5" t="n">
-        <v>334.71</v>
+        <v>40.3</v>
       </c>
       <c r="BB5" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="BC5" t="n">
-        <v>367.1</v>
+        <v>117.6</v>
       </c>
       <c r="BD5" t="n">
         <v>0</v>
       </c>
       <c r="BE5" t="n">
-        <v>40.3</v>
+        <v>0</v>
       </c>
       <c r="BF5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="BG5" t="n">
-        <v>117.6</v>
+        <v>124</v>
       </c>
       <c r="BH5" t="n">
         <v>0</v>
@@ -1710,7 +1710,7 @@
         <v>0</v>
       </c>
       <c r="BK5" t="n">
-        <v>124</v>
+        <v>0</v>
       </c>
       <c r="BL5" t="n">
         <v>0</v>
@@ -1788,7 +1788,7 @@
         <v>32</v>
       </c>
       <c r="I6" t="n">
-        <v>4.94</v>
+        <v>5.27</v>
       </c>
       <c r="J6" t="n">
         <v>31</v>
@@ -1848,7 +1848,7 @@
         <v>70</v>
       </c>
       <c r="AC6" t="n">
-        <v>228.14</v>
+        <v>228.41</v>
       </c>
       <c r="AD6" t="n">
         <v>47</v>
@@ -1863,64 +1863,64 @@
         <v>228.46</v>
       </c>
       <c r="AH6" t="n">
+        <v>52</v>
+      </c>
+      <c r="AI6" t="n">
+        <v>246.41</v>
+      </c>
+      <c r="AJ6" t="n">
         <v>116</v>
       </c>
-      <c r="AI6" t="n">
-        <v>718.6</v>
-      </c>
-      <c r="AJ6" t="n">
+      <c r="AK6" t="n">
+        <v>718.08</v>
+      </c>
+      <c r="AL6" t="n">
         <v>43</v>
       </c>
-      <c r="AK6" t="n">
-        <v>361.3</v>
-      </c>
-      <c r="AL6" t="n">
+      <c r="AM6" t="n">
+        <v>361.83</v>
+      </c>
+      <c r="AN6" t="n">
         <v>16</v>
       </c>
-      <c r="AM6" t="n">
-        <v>178.5</v>
-      </c>
-      <c r="AN6" t="n">
+      <c r="AO6" t="n">
+        <v>178.81</v>
+      </c>
+      <c r="AP6" t="n">
         <v>15</v>
       </c>
-      <c r="AO6" t="n">
-        <v>209.4</v>
-      </c>
-      <c r="AP6" t="n">
-        <v>8</v>
-      </c>
       <c r="AQ6" t="n">
-        <v>142.2</v>
+        <v>209.87</v>
       </c>
       <c r="AR6" t="n">
         <v>8</v>
       </c>
       <c r="AS6" t="n">
-        <v>176.3</v>
+        <v>142.71</v>
       </c>
       <c r="AT6" t="n">
+        <v>8</v>
+      </c>
+      <c r="AU6" t="n">
+        <v>176.19</v>
+      </c>
+      <c r="AV6" t="n">
         <v>3</v>
       </c>
-      <c r="AU6" t="n">
-        <v>81.3</v>
-      </c>
-      <c r="AV6" t="n">
-        <v>2</v>
-      </c>
       <c r="AW6" t="n">
-        <v>66.8</v>
+        <v>81.45</v>
       </c>
       <c r="AX6" t="n">
         <v>2</v>
       </c>
       <c r="AY6" t="n">
-        <v>95.8</v>
+        <v>66.52</v>
       </c>
       <c r="AZ6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BA6" t="n">
-        <v>0</v>
+        <v>95.69</v>
       </c>
       <c r="BB6" t="n">
         <v>0</v>
@@ -1980,7 +1980,7 @@
         <v>1154</v>
       </c>
       <c r="BU6" t="n">
-        <v>3857.18</v>
+        <v>3857.49</v>
       </c>
       <c r="BV6" t="inlineStr">
         <is>

</xml_diff>